<commit_message>
deploy: main → 595b85528506f17c7d0dd052620d7ad733ec88a4
</commit_message>
<xml_diff>
--- a/CodeSystem-diagnosistype-cs.xlsx
+++ b/CodeSystem-diagnosistype-cs.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="44">
   <si>
     <t>Property</t>
   </si>
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://fhir.inera.se/clinicalprocess-healthcond-description/CodeSystem/diagnosistype-cs</t>
+    <t>https://terminologitjansten.inera.se/inera-kodverksforvaltning/kodverk/kv_diagnostyp</t>
   </si>
   <si>
     <t>Version</t>
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>DiagnosisType</t>
+    <t>KV Diagnostyp (fragment)</t>
   </si>
   <si>
     <t>Status</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-01T18:35:17+00:00</t>
+    <t>2026-10-02T11:47:48+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Kodverk för typ av diagnos (huvud- respektive bidiagnos). Definierat i XSD för domänen.</t>
+    <t>Fragment av Ineras kodverk kv_diagnostyp med de koder som används för typ av diagnos i GetDiagnosis (diagnosisBody.typeOfDiagnosis): HD = huvuddiagnos, BY = bidiagnos. Kodverket förvaltas av Inera; detta är en delmängd för validering i IG:n.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -93,6 +93,9 @@
     <t>Case Sensitive</t>
   </si>
   <si>
+    <t>true</t>
+  </si>
+  <si>
     <t>Value Set (all codes)</t>
   </si>
   <si>
@@ -108,7 +111,7 @@
     <t>Content</t>
   </si>
   <si>
-    <t>complete</t>
+    <t>fragment</t>
   </si>
   <si>
     <t>Supplements</t>
@@ -117,9 +120,6 @@
     <t>Count</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>Level</t>
   </si>
   <si>
@@ -135,7 +135,13 @@
     <t>1</t>
   </si>
   <si>
+    <t>HD</t>
+  </si>
+  <si>
     <t>Huvuddiagnos</t>
+  </si>
+  <si>
+    <t>BY</t>
   </si>
   <si>
     <t>Bidiagnos</t>
@@ -389,53 +395,53 @@
       <c r="A15" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="B15" s="2"/>
+      <c r="B15" t="s" s="2">
+        <v>26</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B16" s="2"/>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B17" s="2"/>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B18" s="2"/>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B19" s="2"/>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B21" s="2"/>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>33</v>
-      </c>
-      <c r="B22" t="s" s="2">
         <v>34</v>
       </c>
+      <c r="B22" s="2"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -469,10 +475,10 @@
         <v>40</v>
       </c>
       <c r="C2" t="s" s="2">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3">
@@ -480,13 +486,13 @@
         <v>39</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>